<commit_message>
se corrigio error al consultar ficha
</commit_message>
<xml_diff>
--- a/novedades.xlsx
+++ b/novedades.xlsx
@@ -433,7 +433,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>45371</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="3">
@@ -444,7 +444,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2499992</t>
+          <t>2041211</t>
         </is>
       </c>
     </row>
@@ -456,7 +456,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PROGRAMA DE PRUEBA</t>
+          <t>INTEGRACION DE CONTENIDOS DIGITALES.</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>44669</v>
+        <v>45033</v>
       </c>
     </row>
     <row r="7">
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>45490</v>
+        <v>45489</v>
       </c>
     </row>
     <row r="8">
@@ -550,16 +550,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1005163796</v>
+        <v>1096219906</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LINA FERNANDA</t>
+          <t>CHARLES JAVIER</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>LUNA GOMEZ</t>
+          <t>GALO CONTRERAS</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -575,46 +575,46 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1005221000</v>
+        <v>1096240059</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KEVIN DAVID</t>
+          <t>MARIA PAULA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PINILLA ESTEVEZ</t>
+          <t>ARTEAGA CARRILLO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CANCELADO</t>
+          <t>RETIRO VOLUNTARIO</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1096195573</v>
+        <v>1096243733</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SEBASTIAN</t>
+          <t>SHAROLL DANIELA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>FORERO PATIÑO</t>
+          <t>TORRES CHACON</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CANCELADO</t>
+          <t>RETIRO VOLUNTARIO</t>
         </is>
       </c>
     </row>
@@ -625,21 +625,21 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1096248865</v>
+        <v>1102348123</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CLARINYER DE JESUS</t>
+          <t>ELIANA LISETH</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PONCES SANCHEZ</t>
+          <t>PACHECO BARON</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CANCELADO</t>
+          <t>RETIRO VOLUNTARIO</t>
         </is>
       </c>
     </row>
@@ -650,16 +650,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1096251134</v>
+        <v>57299599</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>JOAQUIN ENRIQUE</t>
+          <t>LOURDES MARIA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>HERRERA GONZALEZ</t>
+          <t>OLIVEROS VILLANUEVA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">

</xml_diff>

<commit_message>
Finalice el modulo de asociar empresa con el aprendiz
</commit_message>
<xml_diff>
--- a/novedades.xlsx
+++ b/novedades.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,7 +433,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>45383</v>
+        <v>45384</v>
       </c>
     </row>
     <row r="3">
@@ -444,7 +444,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2041211</t>
+          <t>2824078</t>
         </is>
       </c>
     </row>
@@ -456,7 +456,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>INTEGRACION DE CONTENIDOS DIGITALES.</t>
+          <t>DISEÑO E INTEGRACION DE MULTIMEDIA</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>45033</v>
+        <v>44760</v>
       </c>
     </row>
     <row r="7">
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>45489</v>
+        <v>45124</v>
       </c>
     </row>
     <row r="8">
@@ -550,21 +550,21 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1096219906</v>
+        <v>1005178211</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CHARLES JAVIER</t>
+          <t>JUAN CAMILO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>GALO CONTRERAS</t>
+          <t>DELGADO CARRASCAL</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>RETIRO VOLUNTARIO</t>
+          <t>CERTIFICADO</t>
         </is>
       </c>
     </row>
@@ -575,21 +575,21 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1096240059</v>
+        <v>1005181992</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MARIA PAULA</t>
+          <t>JOHAN</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ARTEAGA CARRILLO</t>
+          <t>VARGAS CALDERIN</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>RETIRO VOLUNTARIO</t>
+          <t>POR CERTIFICAR</t>
         </is>
       </c>
     </row>
@@ -600,21 +600,21 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1096243733</v>
+        <v>1005184329</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SHAROLL DANIELA</t>
+          <t>WILLIAM ANDRES</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>TORRES CHACON</t>
+          <t>LOPEZ RIOS</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>RETIRO VOLUNTARIO</t>
+          <t>CANCELADO</t>
         </is>
       </c>
     </row>
@@ -625,21 +625,21 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1102348123</v>
+        <v>1005185919</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ELIANA LISETH</t>
+          <t>SEBASTIAN</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PACHECO BARON</t>
+          <t>PERTUZ SAMPAYO</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>RETIRO VOLUNTARIO</t>
+          <t>CERTIFICADO</t>
         </is>
       </c>
     </row>
@@ -650,21 +650,321 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>57299599</v>
+        <v>1005220651</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>LOURDES MARIA</t>
+          <t>BRAYAN EDUARDO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>OLIVEROS VILLANUEVA</t>
+          <t>BADILLO HERRERA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>CERTIFICADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1005239745</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SARAY DUVIANA</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>UNRIZA JAIMES</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>CERTIFICADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1005241421</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CLARA LUCIA</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>RUIZ MONSALVE</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>RETIRO VOLUNTARIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1043962939</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>DANNA KAROLAY</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>RESTREPO SOSA</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CERTIFICADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1048457729</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>DAYANA</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>URRUCHURTU NIÑO</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>CERTIFICADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1049019898</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>KAREN YURLEIDY</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MARIN VARGAS</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>RETIRO VOLUNTARIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1087985197</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>GISELL MARIANA</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MARIN LARROTA</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>CERTIFICADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1096184002</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>DANIELA</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>ROJAS BOTELLO</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>CERTIFICADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1096186262</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>KEVIN ANDRES</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>PARADA SUAREZ</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>RETIRO VOLUNTARIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1096189477</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>KAMILA</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>QUINTERO CARREÑO</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>CERTIFICADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1097183074</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MARIA JOSE</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ORTIZ GUIZA</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>CERTIFICADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1144182405</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CAROLAIN</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ABANIS PEREZ</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>CERTIFICADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>63469380</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>VIDA EMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>SANTOS YAIN</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>CERTIFICADO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Se añadio la tabla(clase) Actividades y se completo la tabla Asignaciones con lo que hacia falta segun el diagrama entidad relación
</commit_message>
<xml_diff>
--- a/novedades.xlsx
+++ b/novedades.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,7 +433,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>45385</v>
+        <v>45390</v>
       </c>
     </row>
     <row r="3">
@@ -444,7 +444,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2824078</t>
+          <t>2041211</t>
         </is>
       </c>
     </row>
@@ -456,7 +456,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DISEÑO E INTEGRACION DE MULTIMEDIA</t>
+          <t>INTEGRACION DE CONTENIDOS DIGITALES.</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>44760</v>
+        <v>45033</v>
       </c>
     </row>
     <row r="7">
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>45124</v>
+        <v>45489</v>
       </c>
     </row>
     <row r="8">
@@ -550,21 +550,21 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1005178211</v>
+        <v>1096219906</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>JUAN CAMILO</t>
+          <t>CHARLES JAVIER</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>DELGADO CARRASCAL</t>
+          <t>GALO CONTRERAS</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CERTIFICADO</t>
+          <t>RETIRO VOLUNTARIO</t>
         </is>
       </c>
     </row>
@@ -575,21 +575,21 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1005181992</v>
+        <v>1096240059</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>JOHAN</t>
+          <t>MARIA PAULA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>VARGAS CALDERIN</t>
+          <t>ARTEAGA CARRILLO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>POR CERTIFICAR</t>
+          <t>RETIRO VOLUNTARIO</t>
         </is>
       </c>
     </row>
@@ -600,21 +600,21 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1005184329</v>
+        <v>1096243733</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>WILLIAM ANDRES</t>
+          <t>SHAROLL DANIELA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>LOPEZ RIOS</t>
+          <t>TORRES CHACON</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CANCELADO</t>
+          <t>RETIRO VOLUNTARIO</t>
         </is>
       </c>
     </row>
@@ -625,21 +625,21 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1005185919</v>
+        <v>1102348123</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SEBASTIAN</t>
+          <t>ELIANA LISETH</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PERTUZ SAMPAYO</t>
+          <t>PACHECO BARON</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CERTIFICADO</t>
+          <t>RETIRO VOLUNTARIO</t>
         </is>
       </c>
     </row>
@@ -650,321 +650,21 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1005220651</v>
+        <v>57299599</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BRAYAN EDUARDO</t>
+          <t>LOURDES MARIA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>BADILLO HERRERA</t>
+          <t>OLIVEROS VILLANUEVA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CERTIFICADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>1005239745</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>SARAY DUVIANA</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>UNRIZA JAIMES</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>CERTIFICADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1005241421</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>CLARA LUCIA</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>RUIZ MONSALVE</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
           <t>RETIRO VOLUNTARIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>1043962939</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>DANNA KAROLAY</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>RESTREPO SOSA</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>CERTIFICADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1048457729</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>DAYANA</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>URRUCHURTU NIÑO</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>CERTIFICADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>TI</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1049019898</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>KAREN YURLEIDY</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>MARIN VARGAS</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>RETIRO VOLUNTARIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1087985197</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>GISELL MARIANA</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>MARIN LARROTA</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>CERTIFICADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1096184002</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>DANIELA</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>ROJAS BOTELLO</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>CERTIFICADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>1096186262</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>KEVIN ANDRES</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>PARADA SUAREZ</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>RETIRO VOLUNTARIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>1096189477</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>KAMILA</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>QUINTERO CARREÑO</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>CERTIFICADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1097183074</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>MARIA JOSE</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>ORTIZ GUIZA</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>CERTIFICADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>1144182405</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>CAROLAIN</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>ABANIS PEREZ</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>CERTIFICADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>63469380</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>VIDA EMPERATRIZ</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>SANTOS YAIN</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>CERTIFICADO</t>
         </is>
       </c>
     </row>

</xml_diff>